<commit_message>
fix: 엑셀 보고서 다중 시트 XML 손상 (print_area 제거 + definedNames 안전망)
</commit_message>
<xml_diff>
--- a/excel-template.xlsx
+++ b/excel-template.xlsx
@@ -8,9 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="수정2 시트" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'수정2 시트'!$A$1:$E$28</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>

</xml_diff>